<commit_message>
feat: restore xsignals for drv and enc
</commit_message>
<xml_diff>
--- a/out/miaow-foc-board.xlsx
+++ b/out/miaow-foc-board.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\guoyr\Desktop\foc-hw\out\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C919B74C-453B-4453-8806-36968F65BD08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{0648D331-7A10-43D3-8EBA-59D769497888}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="13716" yWindow="960" windowWidth="16488" windowHeight="13920" xr2:uid="{EBC5D4B1-89BE-4BBB-B581-443B385F2ED6}"/>
+    <workbookView xWindow="13716" yWindow="960" windowWidth="16488" windowHeight="13920" xr2:uid="{4CDA83A7-882C-434A-B181-CF2A03804383}"/>
   </bookViews>
   <sheets>
     <sheet name="miaow-foc-board" sheetId="1" r:id="rId1"/>
@@ -1009,7 +1009,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3FC43F4-BCEC-49CF-AD55-4CA27A324981}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5F5C916D-80B5-4386-A4D4-2EA560229994}">
   <dimension ref="A1:H69"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>

</xml_diff>

<commit_message>
fix: export pad holes to 3d model
</commit_message>
<xml_diff>
--- a/out/miaow-foc-board.xlsx
+++ b/out/miaow-foc-board.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\guoyr\Desktop\foc-hw\out\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0648D331-7A10-43D3-8EBA-59D769497888}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{8B499A45-78BC-4DDF-A9B3-87BED1C7EB8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="13716" yWindow="960" windowWidth="16488" windowHeight="13920" xr2:uid="{4CDA83A7-882C-434A-B181-CF2A03804383}"/>
+    <workbookView xWindow="13716" yWindow="960" windowWidth="16488" windowHeight="13920" xr2:uid="{7AAB9C73-DFBE-4995-B8C9-A1C84B5B1EC5}"/>
   </bookViews>
   <sheets>
     <sheet name="miaow-foc-board" sheetId="1" r:id="rId1"/>
@@ -1009,7 +1009,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5F5C916D-80B5-4386-A4D4-2EA560229994}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9339D540-AEDA-4470-980C-50952399707F}">
   <dimension ref="A1:H69"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>

</xml_diff>